<commit_message>
Update finance ingestion and PYG reconciliation flows
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_consolidado_2026.xlsx
+++ b/output/spreadsheet/pyg_consolidado_2026.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="P&amp;G-CONSOLIDADO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="i-sl" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="i-ltd" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="i-inc" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="fx-rates" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="P&amp;G-TRIMESTRAL" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;G-CONSOLIDADO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i-sl" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i-ltd" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i-inc" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fx-rates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;G-TRIMESTRAL" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -712,7 +712,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Actualizado: 10/04/2026 12:53 h</t>
+          <t>Actualizado: 16/07/2026 04:08 h</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="C4" s="23" t="n">
-        <v>17191.41</v>
+        <v>17203.81</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>4124.64</v>
+        <v>4006.6</v>
       </c>
     </row>
     <row r="11" ht="12" customHeight="1">
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>133633.77</v>
+        <v>141116.09</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -2595,7 +2595,7 @@
         </is>
       </c>
       <c r="C16" s="23" t="n">
-        <v>-2176.46</v>
+        <v>5020.67</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>4034.69</v>
+        <v>3834.74</v>
       </c>
     </row>
     <row r="26" ht="12" customHeight="1">
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="C28" s="23" t="n">
-        <v>149057.08</v>
+        <v>149216.95</v>
       </c>
     </row>
     <row r="29" ht="12" customHeight="1">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>-522.54</v>
+        <v>-2573.81</v>
       </c>
     </row>
     <row r="31" ht="12" customHeight="1">
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="C31" s="23" t="n">
-        <v>4037.39</v>
+        <v>4058.56</v>
       </c>
     </row>
     <row r="32" ht="12" customHeight="1">
@@ -2835,7 +2835,7 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>2753.58</v>
+        <v>2854.46</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1">
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>16086.79</v>
+        <v>16640.32</v>
       </c>
     </row>
     <row r="34" ht="12" customHeight="1">
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="C37" s="23" t="n">
-        <v>4400.57</v>
+        <v>4342.56</v>
       </c>
     </row>
     <row r="38" ht="12" customHeight="1">
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="C40" s="23" t="n">
-        <v>153533.23</v>
+        <v>167421.13</v>
       </c>
     </row>
     <row r="41" ht="12" customHeight="1">
@@ -2985,7 +2985,7 @@
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>-585.21</v>
+        <v>-2464.45</v>
       </c>
     </row>
     <row r="43" ht="12" customHeight="1">
@@ -3000,7 +3000,7 @@
         </is>
       </c>
       <c r="C43" s="23" t="n">
-        <v>5355.88</v>
+        <v>5323.32</v>
       </c>
     </row>
     <row r="44" ht="12" customHeight="1">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="C44" s="23" t="n">
-        <v>823.08</v>
+        <v>1178.08</v>
       </c>
     </row>
     <row r="45" ht="12" customHeight="1">
@@ -3026,11 +3026,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>diferencias_divisas</t>
         </is>
       </c>
       <c r="C45" s="23" t="n">
-        <v>948.47</v>
+        <v>140.18</v>
       </c>
     </row>
     <row r="46" ht="12" customHeight="1">
@@ -3041,11 +3041,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>shopify</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C46" s="23" t="n">
-        <v>55325.41</v>
+        <v>16518.07</v>
       </c>
     </row>
     <row r="47" ht="12" customHeight="1">
@@ -3056,11 +3056,611 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="n">
+        <v>54733.64</v>
+      </c>
+    </row>
+    <row r="48" ht="12" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="n">
+        <v>49203.02</v>
+      </c>
+    </row>
+    <row r="49" ht="12" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>marketplaces</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="n">
+        <v>1683.63</v>
+      </c>
+    </row>
+    <row r="50" ht="12" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>otros_gastos</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="n">
+        <v>935.45</v>
+      </c>
+    </row>
+    <row r="51" ht="12" customHeight="1">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>otros_ingresos</t>
+        </is>
+      </c>
+      <c r="C51" s="23" t="n">
+        <v>67.09999999999999</v>
+      </c>
+    </row>
+    <row r="52" ht="12" customHeight="1">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="n">
+        <v>3797.02</v>
+      </c>
+    </row>
+    <row r="53" ht="12" customHeight="1">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>royalties</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="n">
+        <v>13605</v>
+      </c>
+    </row>
+    <row r="54" ht="12" customHeight="1">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="n">
+        <v>142754.64</v>
+      </c>
+    </row>
+    <row r="55" ht="12" customHeight="1">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="n">
+        <v>15515.1</v>
+      </c>
+    </row>
+    <row r="56" ht="12" customHeight="1">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>supplies</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="n">
+        <v>-2141.38</v>
+      </c>
+    </row>
+    <row r="57" ht="12" customHeight="1">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>202604</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>technology</t>
         </is>
       </c>
-      <c r="C47" s="23" t="n">
-        <v>163.1</v>
+      <c r="C57" s="23" t="n">
+        <v>5388.18</v>
+      </c>
+    </row>
+    <row r="58" ht="12" customHeight="1">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="n">
+        <v>1083.38</v>
+      </c>
+    </row>
+    <row r="59" ht="12" customHeight="1">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="n">
+        <v>16680.21</v>
+      </c>
+    </row>
+    <row r="60" ht="12" customHeight="1">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="n">
+        <v>50365.6</v>
+      </c>
+    </row>
+    <row r="61" ht="12" customHeight="1">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="n">
+        <v>48654.25</v>
+      </c>
+    </row>
+    <row r="62" ht="12" customHeight="1">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>marketplaces</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="n">
+        <v>-42.49</v>
+      </c>
+    </row>
+    <row r="63" ht="12" customHeight="1">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="n">
+        <v>3753.11</v>
+      </c>
+    </row>
+    <row r="64" ht="12" customHeight="1">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>royalties</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="n">
+        <v>13698</v>
+      </c>
+    </row>
+    <row r="65" ht="12" customHeight="1">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="n">
+        <v>137777.97</v>
+      </c>
+    </row>
+    <row r="66" ht="12" customHeight="1">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="n">
+        <v>15515.1</v>
+      </c>
+    </row>
+    <row r="67" ht="12" customHeight="1">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>supplies</t>
+        </is>
+      </c>
+      <c r="C67" s="23" t="n">
+        <v>-1978.99</v>
+      </c>
+    </row>
+    <row r="68" ht="12" customHeight="1">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>202605</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="C68" s="23" t="n">
+        <v>5671.14</v>
+      </c>
+    </row>
+    <row r="69" ht="12" customHeight="1">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C69" s="23" t="n">
+        <v>998.08</v>
+      </c>
+    </row>
+    <row r="70" ht="12" customHeight="1">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="C70" s="23" t="n">
+        <v>14333.23</v>
+      </c>
+    </row>
+    <row r="71" ht="12" customHeight="1">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C71" s="23" t="n">
+        <v>43073.99</v>
+      </c>
+    </row>
+    <row r="72" ht="12" customHeight="1">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C72" s="23" t="n">
+        <v>46014.43</v>
+      </c>
+    </row>
+    <row r="73" ht="12" customHeight="1">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>marketplaces</t>
+        </is>
+      </c>
+      <c r="C73" s="23" t="n">
+        <v>8690.639999999999</v>
+      </c>
+    </row>
+    <row r="74" ht="12" customHeight="1">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C74" s="23" t="n">
+        <v>3253.12</v>
+      </c>
+    </row>
+    <row r="75" ht="12" customHeight="1">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>royalties</t>
+        </is>
+      </c>
+      <c r="C75" s="23" t="n">
+        <v>11562</v>
+      </c>
+    </row>
+    <row r="76" ht="12" customHeight="1">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C76" s="23" t="n">
+        <v>130750.87</v>
+      </c>
+    </row>
+    <row r="77" ht="12" customHeight="1">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="C77" s="23" t="n">
+        <v>15421.77</v>
+      </c>
+    </row>
+    <row r="78" ht="12" customHeight="1">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>supplies</t>
+        </is>
+      </c>
+      <c r="C78" s="23" t="n">
+        <v>-1396.66</v>
+      </c>
+    </row>
+    <row r="79" ht="12" customHeight="1">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="C79" s="23" t="n">
+        <v>5677.85</v>
+      </c>
+    </row>
+    <row r="80" ht="12" customHeight="1">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C80" s="23" t="n">
+        <v>823.08</v>
+      </c>
+    </row>
+    <row r="81" ht="12" customHeight="1">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="C81" s="23" t="n">
+        <v>-569.03</v>
+      </c>
+    </row>
+    <row r="82" ht="12" customHeight="1">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C82" s="23" t="n">
+        <v>9495.780000000001</v>
+      </c>
+    </row>
+    <row r="83" ht="12" customHeight="1">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C83" s="23" t="n">
+        <v>1942.52</v>
+      </c>
+    </row>
+    <row r="84" ht="12" customHeight="1">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C84" s="23" t="n">
+        <v>70326.75999999999</v>
+      </c>
+    </row>
+    <row r="85" ht="12" customHeight="1">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="C85" s="23" t="n">
+        <v>15515.1</v>
+      </c>
+    </row>
+    <row r="86" ht="12" customHeight="1">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>supplies</t>
+        </is>
+      </c>
+      <c r="C86" s="23" t="n">
+        <v>215.08</v>
+      </c>
+    </row>
+    <row r="87" ht="12" customHeight="1">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="C87" s="23" t="n">
+        <v>1167.66</v>
       </c>
     </row>
   </sheetData>
@@ -3074,7 +3674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3171,7 +3771,7 @@
         </is>
       </c>
       <c r="C6" s="23" t="n">
-        <v>15702.66</v>
+        <v>15649.32</v>
       </c>
     </row>
     <row r="7" ht="12" customHeight="1">
@@ -3246,7 +3846,7 @@
         </is>
       </c>
       <c r="C11" s="23" t="n">
-        <v>19429.25</v>
+        <v>19257.61</v>
       </c>
     </row>
     <row r="12" ht="12" customHeight="1">
@@ -3261,7 +3861,7 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>254.17</v>
+        <v>185.17</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -3291,7 +3891,7 @@
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>9601.129999999999</v>
+        <v>10312</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -3302,11 +3902,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>otros_gastos</t>
         </is>
       </c>
       <c r="C15" s="23" t="n">
-        <v>564.5</v>
+        <v>14.87</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1">
@@ -3317,11 +3917,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>product_sales</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C16" s="23" t="n">
-        <v>22362.26</v>
+        <v>564.5</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -3332,26 +3932,26 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>technology</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>141.32</v>
+        <v>21790.3</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
-          <t>202604</t>
+          <t>202603</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>technology</t>
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>1035.17</v>
+        <v>141.32</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -3362,11 +3962,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
-        <v>284.82</v>
+        <v>185.17</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -3377,11 +3977,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>117.4</v>
+        <v>1911.85</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -3392,92 +3992,92 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>product_sales</t>
+          <t>manufacturing</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>5572.05</v>
+        <v>9507.43</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
-          <t>202605</t>
+          <t>202604</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>185.17</v>
+        <v>492.78</v>
       </c>
     </row>
     <row r="23" ht="12" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>202605</t>
+          <t>202604</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>0</v>
+        <v>18436.42</v>
       </c>
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>202606</t>
+          <t>202604</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>technology</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
-        <v>185.17</v>
+        <v>70.48999999999999</v>
       </c>
     </row>
     <row r="25" ht="12" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>202606</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>0</v>
+        <v>185.17</v>
       </c>
     </row>
     <row r="26" ht="12" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>202607</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>185.17</v>
+        <v>1842.92</v>
       </c>
     </row>
     <row r="27" ht="12" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
-          <t>202607</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3486,88 +4086,88 @@
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>0</v>
+        <v>9150.040000000001</v>
       </c>
     </row>
     <row r="28" ht="12" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>202608</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
-        <v>185.17</v>
+        <v>501.87</v>
       </c>
     </row>
     <row r="29" ht="12" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>202608</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
-        <v>0</v>
+        <v>19826.63</v>
       </c>
     </row>
     <row r="30" ht="12" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>202609</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>technology</t>
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>185.17</v>
+        <v>70.56999999999999</v>
       </c>
     </row>
     <row r="31" ht="12" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
-          <t>202609</t>
+          <t>202606</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C31" s="23" t="n">
-        <v>0</v>
+        <v>185.17</v>
       </c>
     </row>
     <row r="32" ht="12" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>202610</t>
+          <t>202606</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>185.17</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
-          <t>202610</t>
+          <t>202606</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3576,66 +4176,261 @@
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>0</v>
+        <v>4282.62</v>
       </c>
     </row>
     <row r="34" ht="12" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
-          <t>202611</t>
+          <t>202606</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>185.17</v>
+        <v>501.86</v>
       </c>
     </row>
     <row r="35" ht="12" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
-          <t>202611</t>
+          <t>202606</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>0</v>
+        <v>20562.26</v>
       </c>
     </row>
     <row r="36" ht="12" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
-          <t>202612</t>
+          <t>202606</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>technology</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
-        <v>185.17</v>
+        <v>70.12</v>
       </c>
     </row>
     <row r="37" ht="12" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="38" ht="12" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>1176.14</v>
+      </c>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="n">
+        <v>220.7</v>
+      </c>
+    </row>
+    <row r="40" ht="12" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>product_sales</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="n">
+        <v>9133.639999999999</v>
+      </c>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="42" ht="12" customHeight="1">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="12" customHeight="1">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="44" ht="12" customHeight="1">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="12" customHeight="1">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="46" ht="12" customHeight="1">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="12" customHeight="1">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>202611</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="48" ht="12" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>202611</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="12" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>202612</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="50" ht="12" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>202612</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>manufacturing</t>
         </is>
       </c>
-      <c r="C37" s="23" t="n">
+      <c r="C50" s="23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3650,7 +4445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3717,7 +4512,7 @@
         </is>
       </c>
       <c r="C4" s="23" t="n">
-        <v>4663.04</v>
+        <v>4789.72</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -3747,7 +4542,7 @@
         </is>
       </c>
       <c r="C6" s="23" t="n">
-        <v>10261.58</v>
+        <v>10286.53</v>
       </c>
     </row>
     <row r="7" ht="12" customHeight="1">
@@ -3762,7 +4557,7 @@
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>1332.48</v>
+        <v>1316.39</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
@@ -3792,7 +4587,7 @@
         </is>
       </c>
       <c r="C9" s="23" t="n">
-        <v>5066.36</v>
+        <v>5220.72</v>
       </c>
     </row>
     <row r="10" ht="12" customHeight="1">
@@ -3822,7 +4617,7 @@
         </is>
       </c>
       <c r="C11" s="23" t="n">
-        <v>15549.06</v>
+        <v>15189.15</v>
       </c>
     </row>
     <row r="12" ht="12" customHeight="1">
@@ -3837,7 +4632,7 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>1409.68</v>
+        <v>1474.77</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -3848,11 +4643,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C13" s="23" t="n">
-        <v>2767.57</v>
+        <v>4826.94</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1">
@@ -3863,11 +4658,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>manufacturing</t>
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>520.41</v>
+        <v>6286.98</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -3878,26 +4673,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>product_sales</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C15" s="23" t="n">
-        <v>16536.75</v>
+        <v>520.41</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
-          <t>202604</t>
+          <t>202603</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C16" s="23" t="n">
-        <v>1257</v>
+        <v>16690.76</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -3908,11 +4703,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>67.3</v>
+        <v>1402.69</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
@@ -3923,11 +4718,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>101</v>
+        <v>2945.34</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -3938,77 +4733,77 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>product_sales</t>
+          <t>manufacturing</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
-        <v>4493.94</v>
+        <v>4815.93</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
-          <t>202605</t>
+          <t>202604</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>0</v>
+        <v>466.64</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
-          <t>202606</t>
+          <t>202604</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>0</v>
+        <v>15746.89</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
-          <t>202607</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>0</v>
+        <v>1302.88</v>
       </c>
     </row>
     <row r="23" ht="12" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>202608</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>0</v>
+        <v>2254.01</v>
       </c>
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>202609</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4017,51 +4812,246 @@
         </is>
       </c>
       <c r="C24" s="23" t="n">
-        <v>0</v>
+        <v>2661.73</v>
       </c>
     </row>
     <row r="25" ht="12" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>202610</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>0</v>
+        <v>362.95</v>
       </c>
     </row>
     <row r="26" ht="12" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>202611</t>
+          <t>202605</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>0</v>
+        <v>13016.46</v>
       </c>
     </row>
     <row r="27" ht="12" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>1281.29</v>
+      </c>
+    </row>
+    <row r="28" ht="12" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>2614.92</v>
+      </c>
+    </row>
+    <row r="29" ht="12" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>5277.94</v>
+      </c>
+    </row>
+    <row r="30" ht="12" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>474.77</v>
+      </c>
+    </row>
+    <row r="31" ht="12" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>202606</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>product_sales</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>17387.52</v>
+      </c>
+    </row>
+    <row r="32" ht="12" customHeight="1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="33" ht="12" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n">
+        <v>140.54</v>
+      </c>
+    </row>
+    <row r="34" ht="12" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>134.45</v>
+      </c>
+    </row>
+    <row r="35" ht="12" customHeight="1">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>product_sales</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>4147.97</v>
+      </c>
+    </row>
+    <row r="36" ht="12" customHeight="1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" ht="12" customHeight="1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" ht="12" customHeight="1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" ht="12" customHeight="1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>202611</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" ht="12" customHeight="1">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>202612</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>manufacturing</t>
         </is>
       </c>
-      <c r="C27" s="23" t="n">
+      <c r="C40" s="23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4203,7 +5193,7 @@
         </is>
       </c>
       <c r="C8" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.86625</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -4218,7 +5208,7 @@
         </is>
       </c>
       <c r="C9" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1702</v>
       </c>
     </row>
     <row r="10" ht="12" customHeight="1">
@@ -4233,7 +5223,7 @@
         </is>
       </c>
       <c r="C10" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.8672299999999999</v>
       </c>
     </row>
     <row r="11" ht="12" customHeight="1">
@@ -4248,7 +5238,7 @@
         </is>
       </c>
       <c r="C11" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1644</v>
       </c>
     </row>
     <row r="12" ht="12" customHeight="1">
@@ -4263,7 +5253,7 @@
         </is>
       </c>
       <c r="C12" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.86178</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -4278,7 +5268,7 @@
         </is>
       </c>
       <c r="C13" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1394</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1">
@@ -4293,7 +5283,7 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.85093</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -4308,7 +5298,7 @@
         </is>
       </c>
       <c r="C15" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1406</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1">
@@ -4323,7 +5313,7 @@
         </is>
       </c>
       <c r="C16" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.85093</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -4338,7 +5328,7 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1406</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
@@ -4353,7 +5343,7 @@
         </is>
       </c>
       <c r="C18" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.85093</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -4368,7 +5358,7 @@
         </is>
       </c>
       <c r="C19" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1406</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -4383,7 +5373,7 @@
         </is>
       </c>
       <c r="C20" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.85093</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -4398,7 +5388,7 @@
         </is>
       </c>
       <c r="C21" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1406</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
@@ -4413,7 +5403,7 @@
         </is>
       </c>
       <c r="C22" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.85093</v>
       </c>
     </row>
     <row r="23" ht="12" customHeight="1">
@@ -4428,7 +5418,7 @@
         </is>
       </c>
       <c r="C23" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1406</v>
       </c>
     </row>
     <row r="24" ht="12" customHeight="1">
@@ -4443,7 +5433,7 @@
         </is>
       </c>
       <c r="C24" s="24" t="n">
-        <v>0.87053</v>
+        <v>0.85093</v>
       </c>
     </row>
     <row r="25" ht="12" customHeight="1">
@@ -4458,7 +5448,7 @@
         </is>
       </c>
       <c r="C25" s="24" t="n">
-        <v>1.1685</v>
+        <v>1.1406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Phoenix cleaning provider and invoice
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_consolidado_2026.xlsx
+++ b/output/spreadsheet/pyg_consolidado_2026.xlsx
@@ -724,7 +724,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Shopify daily average | Actualizado: 31/07/2026 09:55 h</t>
+          <t>Shopify daily average | Actualizado: 04/09/2026 10:00 h</t>
         </is>
       </c>
       <c r="D3">
@@ -2785,7 +2785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C165"/>
+  <dimension ref="A1:C208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="C14" s="25" t="n">
-        <v>132906.22</v>
+        <v>133035.43</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="C15" s="25" t="n">
-        <v>5472.24</v>
+        <v>5482.24</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>20230.26</v>
+        <v>20271.04</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>61194.44</v>
+        <v>61194.43</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -3092,7 +3092,7 @@
         </is>
       </c>
       <c r="C20" s="25" t="n">
-        <v>25562.13</v>
+        <v>25590.34</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="C21" s="25" t="n">
-        <v>18488.36</v>
+        <v>18538.59</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="C39" s="25" t="n">
-        <v>148647.56</v>
+        <v>148756.85</v>
       </c>
     </row>
     <row r="40" ht="12" customHeight="1">
@@ -3392,7 +3392,7 @@
         </is>
       </c>
       <c r="C40" s="25" t="n">
-        <v>6064.69</v>
+        <v>6077.94</v>
       </c>
     </row>
     <row r="41" ht="12" customHeight="1">
@@ -3422,7 +3422,7 @@
         </is>
       </c>
       <c r="C42" s="25" t="n">
-        <v>19166.62</v>
+        <v>19196.42</v>
       </c>
     </row>
     <row r="43" ht="12" customHeight="1">
@@ -3452,7 +3452,7 @@
         </is>
       </c>
       <c r="C44" s="25" t="n">
-        <v>73214.46000000001</v>
+        <v>73214.47</v>
       </c>
     </row>
     <row r="45" ht="12" customHeight="1">
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="C45" s="25" t="n">
-        <v>27467.98</v>
+        <v>27502.63</v>
       </c>
     </row>
     <row r="46" ht="12" customHeight="1">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="C47" s="25" t="n">
-        <v>20013.28</v>
+        <v>20044.86</v>
       </c>
     </row>
     <row r="48" ht="12" customHeight="1">
@@ -3722,7 +3722,7 @@
         </is>
       </c>
       <c r="C62" s="25" t="n">
-        <v>153013.84</v>
+        <v>153156.89</v>
       </c>
     </row>
     <row r="63" ht="12" customHeight="1">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="C63" s="25" t="n">
-        <v>5410.61</v>
+        <v>5428.11</v>
       </c>
     </row>
     <row r="64" ht="12" customHeight="1">
@@ -3767,7 +3767,7 @@
         </is>
       </c>
       <c r="C65" s="25" t="n">
-        <v>24820.62</v>
+        <v>24871.75</v>
       </c>
     </row>
     <row r="66" ht="12" customHeight="1">
@@ -3782,7 +3782,7 @@
         </is>
       </c>
       <c r="C66" s="25" t="n">
-        <v>70845.75</v>
+        <v>70845.74000000001</v>
       </c>
     </row>
     <row r="67" ht="12" customHeight="1">
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="C67" s="25" t="n">
-        <v>31210.51</v>
+        <v>31270.44</v>
       </c>
     </row>
     <row r="68" ht="12" customHeight="1">
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="C69" s="25" t="n">
-        <v>20244.06</v>
+        <v>20258.56</v>
       </c>
     </row>
     <row r="70" ht="12" customHeight="1">
@@ -4067,7 +4067,7 @@
         </is>
       </c>
       <c r="C85" s="25" t="n">
-        <v>143315.27</v>
+        <v>143535.6</v>
       </c>
     </row>
     <row r="86" ht="12" customHeight="1">
@@ -4082,7 +4082,7 @@
         </is>
       </c>
       <c r="C86" s="25" t="n">
-        <v>4085.09</v>
+        <v>4107.27</v>
       </c>
     </row>
     <row r="87" ht="12" customHeight="1">
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="C87" s="25" t="n">
-        <v>151.72</v>
+        <v>159.19</v>
       </c>
     </row>
     <row r="88" ht="12" customHeight="1">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="C88" s="25" t="n">
-        <v>19303.41</v>
+        <v>19358.29</v>
       </c>
     </row>
     <row r="89" ht="12" customHeight="1">
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="C91" s="25" t="n">
-        <v>27169.89</v>
+        <v>27181.78</v>
       </c>
     </row>
     <row r="92" ht="12" customHeight="1">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="C93" s="25" t="n">
-        <v>18345.04</v>
+        <v>18468.95</v>
       </c>
     </row>
     <row r="94" ht="12" customHeight="1">
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="C106" s="25" t="n">
-        <v>138846.78</v>
+        <v>138924.57</v>
       </c>
     </row>
     <row r="107" ht="12" customHeight="1">
@@ -4397,7 +4397,7 @@
         </is>
       </c>
       <c r="C107" s="25" t="n">
-        <v>5461.52</v>
+        <v>5463.67</v>
       </c>
     </row>
     <row r="108" ht="12" customHeight="1">
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="C109" s="25" t="n">
-        <v>16757.78</v>
+        <v>16788.44</v>
       </c>
     </row>
     <row r="110" ht="12" customHeight="1">
@@ -4457,7 +4457,7 @@
         </is>
       </c>
       <c r="C111" s="25" t="n">
-        <v>71605.44</v>
+        <v>71605.42999999999</v>
       </c>
     </row>
     <row r="112" ht="12" customHeight="1">
@@ -4472,7 +4472,7 @@
         </is>
       </c>
       <c r="C112" s="25" t="n">
-        <v>26658.58</v>
+        <v>26689.09</v>
       </c>
     </row>
     <row r="113" ht="12" customHeight="1">
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="C114" s="25" t="n">
-        <v>17195.67</v>
+        <v>17210.15</v>
       </c>
     </row>
     <row r="115" ht="12" customHeight="1">
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="C146" s="25" t="n">
-        <v>2151.49</v>
+        <v>17318.74</v>
       </c>
     </row>
     <row r="147" ht="12" customHeight="1">
@@ -4997,7 +4997,7 @@
         </is>
       </c>
       <c r="C147" s="25" t="n">
-        <v>16290.08</v>
+        <v>55102.78</v>
       </c>
     </row>
     <row r="148" ht="12" customHeight="1">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>marketing</t>
         </is>
       </c>
       <c r="C148" s="25" t="n">
-        <v>4203.31</v>
+        <v>59827.31</v>
       </c>
     </row>
     <row r="149" ht="12" customHeight="1">
@@ -5023,11 +5023,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>shopify</t>
+          <t>marketplaces</t>
         </is>
       </c>
       <c r="C149" s="25" t="n">
-        <v>151803.64</v>
+        <v>1314.69</v>
       </c>
     </row>
     <row r="150" ht="12" customHeight="1">
@@ -5038,11 +5038,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>shopify_at</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C150" s="25" t="n">
-        <v>4831.74</v>
+        <v>4329.19</v>
       </c>
     </row>
     <row r="151" ht="12" customHeight="1">
@@ -5053,11 +5053,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>shopify_be</t>
+          <t>royalties</t>
         </is>
       </c>
       <c r="C151" s="25" t="n">
-        <v>4046.54</v>
+        <v>14826</v>
       </c>
     </row>
     <row r="152" ht="12" customHeight="1">
@@ -5068,11 +5068,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>shopify_cz</t>
+          <t>shopify</t>
         </is>
       </c>
       <c r="C152" s="25" t="n">
-        <v>975.79</v>
+        <v>165237.94</v>
       </c>
     </row>
     <row r="153" ht="12" customHeight="1">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>shopify_de</t>
+          <t>shopify_at</t>
         </is>
       </c>
       <c r="C153" s="25" t="n">
-        <v>17211.56</v>
+        <v>4858.31</v>
       </c>
     </row>
     <row r="154" ht="12" customHeight="1">
@@ -5098,11 +5098,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>shopify_dk</t>
+          <t>shopify_be</t>
         </is>
       </c>
       <c r="C154" s="25" t="n">
-        <v>1650.84</v>
+        <v>4442.82</v>
       </c>
     </row>
     <row r="155" ht="12" customHeight="1">
@@ -5113,11 +5113,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>shopify_es</t>
+          <t>shopify_cz</t>
         </is>
       </c>
       <c r="C155" s="25" t="n">
-        <v>63672.62</v>
+        <v>975.79</v>
       </c>
     </row>
     <row r="156" ht="12" customHeight="1">
@@ -5128,11 +5128,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>shopify_fr</t>
+          <t>shopify_de</t>
         </is>
       </c>
       <c r="C156" s="25" t="n">
-        <v>29243.18</v>
+        <v>17581.98</v>
       </c>
     </row>
     <row r="157" ht="12" customHeight="1">
@@ -5143,11 +5143,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>shopify_ie</t>
+          <t>shopify_dk</t>
         </is>
       </c>
       <c r="C157" s="25" t="n">
-        <v>142.11</v>
+        <v>1697.61</v>
       </c>
     </row>
     <row r="158" ht="12" customHeight="1">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>shopify_it</t>
+          <t>shopify_es</t>
         </is>
       </c>
       <c r="C158" s="25" t="n">
-        <v>16694.29</v>
+        <v>75419.2</v>
       </c>
     </row>
     <row r="159" ht="12" customHeight="1">
@@ -5173,11 +5173,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>shopify_lu</t>
+          <t>shopify_fr</t>
         </is>
       </c>
       <c r="C159" s="25" t="n">
-        <v>59.79</v>
+        <v>30091.81</v>
       </c>
     </row>
     <row r="160" ht="12" customHeight="1">
@@ -5188,11 +5188,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>shopify_nl</t>
+          <t>shopify_ie</t>
         </is>
       </c>
       <c r="C160" s="25" t="n">
-        <v>2989.75</v>
+        <v>142.11</v>
       </c>
     </row>
     <row r="161" ht="12" customHeight="1">
@@ -5203,11 +5203,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>shopify_pl</t>
+          <t>shopify_it</t>
         </is>
       </c>
       <c r="C161" s="25" t="n">
-        <v>4806.7</v>
+        <v>17113.21</v>
       </c>
     </row>
     <row r="162" ht="12" customHeight="1">
@@ -5218,11 +5218,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>shopify_pt</t>
+          <t>shopify_lu</t>
         </is>
       </c>
       <c r="C162" s="25" t="n">
-        <v>2889.06</v>
+        <v>59.79</v>
       </c>
     </row>
     <row r="163" ht="12" customHeight="1">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>shopify_se</t>
+          <t>shopify_nl</t>
         </is>
       </c>
       <c r="C163" s="25" t="n">
-        <v>2589.67</v>
+        <v>3070.58</v>
       </c>
     </row>
     <row r="164" ht="12" customHeight="1">
@@ -5248,11 +5248,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>shopify_pl</t>
         </is>
       </c>
       <c r="C164" s="25" t="n">
-        <v>15515.1</v>
+        <v>4336.45</v>
       </c>
     </row>
     <row r="165" ht="12" customHeight="1">
@@ -5263,11 +5263,656 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
+          <t>shopify_pt</t>
+        </is>
+      </c>
+      <c r="C165" s="25" t="n">
+        <v>3046.3</v>
+      </c>
+    </row>
+    <row r="166" ht="12" customHeight="1">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>shopify_se</t>
+        </is>
+      </c>
+      <c r="C166" s="25" t="n">
+        <v>2401.98</v>
+      </c>
+    </row>
+    <row r="167" ht="12" customHeight="1">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="C167" s="25" t="n">
+        <v>15515.1</v>
+      </c>
+    </row>
+    <row r="168" ht="12" customHeight="1">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>202607</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
           <t>technology</t>
         </is>
       </c>
-      <c r="C165" s="25" t="n">
-        <v>4640.58</v>
+      <c r="C168" s="25" t="n">
+        <v>5820.83</v>
+      </c>
+    </row>
+    <row r="169" ht="12" customHeight="1">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C169" s="25" t="n">
+        <v>3591.17</v>
+      </c>
+    </row>
+    <row r="170" ht="12" customHeight="1">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>logistics</t>
+        </is>
+      </c>
+      <c r="C170" s="25" t="n">
+        <v>5945.7</v>
+      </c>
+    </row>
+    <row r="171" ht="12" customHeight="1">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C171" s="25" t="n">
+        <v>53033.35</v>
+      </c>
+    </row>
+    <row r="172" ht="12" customHeight="1">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C172" s="25" t="n">
+        <v>70686.05</v>
+      </c>
+    </row>
+    <row r="173" ht="12" customHeight="1">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C173" s="25" t="n">
+        <v>5420.92</v>
+      </c>
+    </row>
+    <row r="174" ht="12" customHeight="1">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>royalties</t>
+        </is>
+      </c>
+      <c r="C174" s="25" t="n">
+        <v>17256</v>
+      </c>
+    </row>
+    <row r="175" ht="12" customHeight="1">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C175" s="25" t="n">
+        <v>177948.1</v>
+      </c>
+    </row>
+    <row r="176" ht="12" customHeight="1">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>shopify_at</t>
+        </is>
+      </c>
+      <c r="C176" s="25" t="n">
+        <v>5384.02</v>
+      </c>
+    </row>
+    <row r="177" ht="12" customHeight="1">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>shopify_be</t>
+        </is>
+      </c>
+      <c r="C177" s="25" t="n">
+        <v>5783.04</v>
+      </c>
+    </row>
+    <row r="178" ht="12" customHeight="1">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>shopify_cz</t>
+        </is>
+      </c>
+      <c r="C178" s="25" t="n">
+        <v>2748.7</v>
+      </c>
+    </row>
+    <row r="179" ht="12" customHeight="1">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>shopify_de</t>
+        </is>
+      </c>
+      <c r="C179" s="25" t="n">
+        <v>24151.32</v>
+      </c>
+    </row>
+    <row r="180" ht="12" customHeight="1">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>shopify_dk</t>
+        </is>
+      </c>
+      <c r="C180" s="25" t="n">
+        <v>3637.97</v>
+      </c>
+    </row>
+    <row r="181" ht="12" customHeight="1">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>shopify_es</t>
+        </is>
+      </c>
+      <c r="C181" s="25" t="n">
+        <v>65408.07</v>
+      </c>
+    </row>
+    <row r="182" ht="12" customHeight="1">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>shopify_fr</t>
+        </is>
+      </c>
+      <c r="C182" s="25" t="n">
+        <v>31071.53</v>
+      </c>
+    </row>
+    <row r="183" ht="12" customHeight="1">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>shopify_ie</t>
+        </is>
+      </c>
+      <c r="C183" s="25" t="n">
+        <v>122.02</v>
+      </c>
+    </row>
+    <row r="184" ht="12" customHeight="1">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>shopify_it</t>
+        </is>
+      </c>
+      <c r="C184" s="25" t="n">
+        <v>16806.38</v>
+      </c>
+    </row>
+    <row r="185" ht="12" customHeight="1">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>shopify_lu</t>
+        </is>
+      </c>
+      <c r="C185" s="25" t="n">
+        <v>111.84</v>
+      </c>
+    </row>
+    <row r="186" ht="12" customHeight="1">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>shopify_nl</t>
+        </is>
+      </c>
+      <c r="C186" s="25" t="n">
+        <v>6489.92</v>
+      </c>
+    </row>
+    <row r="187" ht="12" customHeight="1">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>shopify_pl</t>
+        </is>
+      </c>
+      <c r="C187" s="25" t="n">
+        <v>7739.27</v>
+      </c>
+    </row>
+    <row r="188" ht="12" customHeight="1">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>shopify_pt</t>
+        </is>
+      </c>
+      <c r="C188" s="25" t="n">
+        <v>4126.93</v>
+      </c>
+    </row>
+    <row r="189" ht="12" customHeight="1">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>shopify_se</t>
+        </is>
+      </c>
+      <c r="C189" s="25" t="n">
+        <v>4367.09</v>
+      </c>
+    </row>
+    <row r="190" ht="12" customHeight="1">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+      <c r="C190" s="25" t="n">
+        <v>15515.1</v>
+      </c>
+    </row>
+    <row r="191" ht="12" customHeight="1">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="C191" s="25" t="n">
+        <v>5855.58</v>
+      </c>
+    </row>
+    <row r="192" ht="12" customHeight="1">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C192" s="25" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="193" ht="12" customHeight="1">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C193" s="25" t="n">
+        <v>645.91</v>
+      </c>
+    </row>
+    <row r="194" ht="12" customHeight="1">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>shopify</t>
+        </is>
+      </c>
+      <c r="C194" s="25" t="n">
+        <v>20130.13</v>
+      </c>
+    </row>
+    <row r="195" ht="12" customHeight="1">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>shopify_at</t>
+        </is>
+      </c>
+      <c r="C195" s="25" t="n">
+        <v>305.59</v>
+      </c>
+    </row>
+    <row r="196" ht="12" customHeight="1">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>shopify_be</t>
+        </is>
+      </c>
+      <c r="C196" s="25" t="n">
+        <v>379.38</v>
+      </c>
+    </row>
+    <row r="197" ht="12" customHeight="1">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>shopify_cz</t>
+        </is>
+      </c>
+      <c r="C197" s="25" t="n">
+        <v>248.15</v>
+      </c>
+    </row>
+    <row r="198" ht="12" customHeight="1">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>shopify_de</t>
+        </is>
+      </c>
+      <c r="C198" s="25" t="n">
+        <v>1796.77</v>
+      </c>
+    </row>
+    <row r="199" ht="12" customHeight="1">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>shopify_dk</t>
+        </is>
+      </c>
+      <c r="C199" s="25" t="n">
+        <v>369.04</v>
+      </c>
+    </row>
+    <row r="200" ht="12" customHeight="1">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>shopify_es</t>
+        </is>
+      </c>
+      <c r="C200" s="25" t="n">
+        <v>7567.43</v>
+      </c>
+    </row>
+    <row r="201" ht="12" customHeight="1">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>shopify_fr</t>
+        </is>
+      </c>
+      <c r="C201" s="25" t="n">
+        <v>4375.88</v>
+      </c>
+    </row>
+    <row r="202" ht="12" customHeight="1">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>shopify_it</t>
+        </is>
+      </c>
+      <c r="C202" s="25" t="n">
+        <v>1985.8</v>
+      </c>
+    </row>
+    <row r="203" ht="12" customHeight="1">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>shopify_lu</t>
+        </is>
+      </c>
+      <c r="C203" s="25" t="n">
+        <v>71.34999999999999</v>
+      </c>
+    </row>
+    <row r="204" ht="12" customHeight="1">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>shopify_nl</t>
+        </is>
+      </c>
+      <c r="C204" s="25" t="n">
+        <v>1084.32</v>
+      </c>
+    </row>
+    <row r="205" ht="12" customHeight="1">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>shopify_pl</t>
+        </is>
+      </c>
+      <c r="C205" s="25" t="n">
+        <v>705.03</v>
+      </c>
+    </row>
+    <row r="206" ht="12" customHeight="1">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>shopify_pt</t>
+        </is>
+      </c>
+      <c r="C206" s="25" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="207" ht="12" customHeight="1">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>shopify_se</t>
+        </is>
+      </c>
+      <c r="C207" s="25" t="n">
+        <v>749.39</v>
+      </c>
+    </row>
+    <row r="208" ht="12" customHeight="1">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="C208" s="25" t="n">
+        <v>106.35</v>
       </c>
     </row>
   </sheetData>
@@ -5281,7 +5926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5348,7 +5993,7 @@
         </is>
       </c>
       <c r="C4" s="25" t="n">
-        <v>8005.88</v>
+        <v>7985.13</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -5378,7 +6023,7 @@
         </is>
       </c>
       <c r="C6" s="25" t="n">
-        <v>15834.87</v>
+        <v>15702.66</v>
       </c>
     </row>
     <row r="7" ht="12" customHeight="1">
@@ -5393,7 +6038,7 @@
         </is>
       </c>
       <c r="C7" s="25" t="n">
-        <v>15834.87</v>
+        <v>15702.66</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
@@ -5438,7 +6083,7 @@
         </is>
       </c>
       <c r="C10" s="25" t="n">
-        <v>8128.95</v>
+        <v>8101.87</v>
       </c>
     </row>
     <row r="11" ht="12" customHeight="1">
@@ -5528,7 +6173,7 @@
         </is>
       </c>
       <c r="C16" s="25" t="n">
-        <v>10288.42</v>
+        <v>10276.8</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -5573,7 +6218,7 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>22434.6</v>
+        <v>22362.26</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -5588,7 +6233,7 @@
         </is>
       </c>
       <c r="C20" s="25" t="n">
-        <v>22434.6</v>
+        <v>22362.26</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -5648,7 +6293,7 @@
         </is>
       </c>
       <c r="C24" s="25" t="n">
-        <v>9461.92</v>
+        <v>9462.610000000001</v>
       </c>
     </row>
     <row r="25" ht="12" customHeight="1">
@@ -5678,7 +6323,7 @@
         </is>
       </c>
       <c r="C26" s="25" t="n">
-        <v>18428.09</v>
+        <v>18321.91</v>
       </c>
     </row>
     <row r="27" ht="12" customHeight="1">
@@ -5693,7 +6338,7 @@
         </is>
       </c>
       <c r="C27" s="25" t="n">
-        <v>18428.09</v>
+        <v>18321.91</v>
       </c>
     </row>
     <row r="28" ht="12" customHeight="1">
@@ -5753,7 +6398,7 @@
         </is>
       </c>
       <c r="C31" s="25" t="n">
-        <v>9098.82</v>
+        <v>9150.040000000001</v>
       </c>
     </row>
     <row r="32" ht="12" customHeight="1">
@@ -5783,7 +6428,7 @@
         </is>
       </c>
       <c r="C33" s="25" t="n">
-        <v>19722.14</v>
+        <v>19784.52</v>
       </c>
     </row>
     <row r="34" ht="12" customHeight="1">
@@ -5798,7 +6443,7 @@
         </is>
       </c>
       <c r="C34" s="25" t="n">
-        <v>19722.14</v>
+        <v>19784.52</v>
       </c>
     </row>
     <row r="35" ht="12" customHeight="1">
@@ -5858,7 +6503,7 @@
         </is>
       </c>
       <c r="C38" s="25" t="n">
-        <v>4310.6</v>
+        <v>4282.62</v>
       </c>
     </row>
     <row r="39" ht="12" customHeight="1">
@@ -5888,7 +6533,7 @@
         </is>
       </c>
       <c r="C40" s="25" t="n">
-        <v>20311</v>
+        <v>20286.92</v>
       </c>
     </row>
     <row r="41" ht="12" customHeight="1">
@@ -5903,7 +6548,7 @@
         </is>
       </c>
       <c r="C41" s="25" t="n">
-        <v>20311</v>
+        <v>20286.92</v>
       </c>
     </row>
     <row r="42" ht="12" customHeight="1">
@@ -5948,7 +6593,7 @@
         </is>
       </c>
       <c r="C44" s="25" t="n">
-        <v>2111.42</v>
+        <v>2934.99</v>
       </c>
     </row>
     <row r="45" ht="12" customHeight="1">
@@ -5963,7 +6608,7 @@
         </is>
       </c>
       <c r="C45" s="25" t="n">
-        <v>446.24</v>
+        <v>465.69</v>
       </c>
     </row>
     <row r="46" ht="12" customHeight="1">
@@ -5978,7 +6623,7 @@
         </is>
       </c>
       <c r="C46" s="25" t="n">
-        <v>18341.96</v>
+        <v>19044.11</v>
       </c>
     </row>
     <row r="47" ht="12" customHeight="1">
@@ -5993,22 +6638,22 @@
         </is>
       </c>
       <c r="C47" s="25" t="n">
-        <v>18341.96</v>
+        <v>19044.11</v>
       </c>
     </row>
     <row r="48" ht="12" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
-          <t>202608</t>
+          <t>202607</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>technology</t>
         </is>
       </c>
       <c r="C48" s="25" t="n">
-        <v>185.17</v>
+        <v>69.63</v>
       </c>
     </row>
     <row r="49" ht="12" customHeight="1">
@@ -6019,77 +6664,77 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C49" s="25" t="n">
-        <v>0</v>
+        <v>185.17</v>
       </c>
     </row>
     <row r="50" ht="12" customHeight="1">
       <c r="A50" t="inlineStr">
         <is>
-          <t>202609</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>manufacturing</t>
         </is>
       </c>
       <c r="C50" s="25" t="n">
-        <v>185.17</v>
+        <v>1934.46</v>
       </c>
     </row>
     <row r="51" ht="12" customHeight="1">
       <c r="A51" t="inlineStr">
         <is>
-          <t>202609</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C51" s="25" t="n">
-        <v>0</v>
+        <v>493.74</v>
       </c>
     </row>
     <row r="52" ht="12" customHeight="1">
       <c r="A52" t="inlineStr">
         <is>
-          <t>202610</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C52" s="25" t="n">
-        <v>185.17</v>
+        <v>19560</v>
       </c>
     </row>
     <row r="53" ht="12" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
-          <t>202610</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>shopify_gb</t>
         </is>
       </c>
       <c r="C53" s="25" t="n">
-        <v>0</v>
+        <v>19560</v>
       </c>
     </row>
     <row r="54" ht="12" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t>202611</t>
+          <t>202609</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6104,7 +6749,7 @@
     <row r="55" ht="12" customHeight="1">
       <c r="A55" t="inlineStr">
         <is>
-          <t>202611</t>
+          <t>202609</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6113,36 +6758,141 @@
         </is>
       </c>
       <c r="C55" s="25" t="n">
-        <v>0</v>
+        <v>281.03</v>
       </c>
     </row>
     <row r="56" ht="12" customHeight="1">
       <c r="A56" t="inlineStr">
         <is>
-          <t>202612</t>
+          <t>202609</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C56" s="25" t="n">
-        <v>185.17</v>
+        <v>59.74</v>
       </c>
     </row>
     <row r="57" ht="12" customHeight="1">
       <c r="A57" t="inlineStr">
         <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>product_sales</t>
+        </is>
+      </c>
+      <c r="C57" s="25" t="n">
+        <v>2558.94</v>
+      </c>
+    </row>
+    <row r="58" ht="12" customHeight="1">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>shopify_gb</t>
+        </is>
+      </c>
+      <c r="C58" s="25" t="n">
+        <v>2558.94</v>
+      </c>
+    </row>
+    <row r="59" ht="12" customHeight="1">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C59" s="25" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="60" ht="12" customHeight="1">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C60" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" ht="12" customHeight="1">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>202611</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C61" s="25" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="62" ht="12" customHeight="1">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>202611</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C62" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="12" customHeight="1">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>202612</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C63" s="25" t="n">
+        <v>185.17</v>
+      </c>
+    </row>
+    <row r="64" ht="12" customHeight="1">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>202612</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>manufacturing</t>
         </is>
       </c>
-      <c r="C57" s="25" t="n">
+      <c r="C64" s="25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6157,7 +6907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6745,11 +7495,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C39" s="25" t="n">
-        <v>434.04</v>
+        <v>2236.13</v>
       </c>
     </row>
     <row r="40" ht="12" customHeight="1">
@@ -6760,11 +7510,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>payment_fees</t>
+          <t>manufacturing</t>
         </is>
       </c>
       <c r="C40" s="25" t="n">
-        <v>354.62</v>
+        <v>3194.56</v>
       </c>
     </row>
     <row r="41" ht="12" customHeight="1">
@@ -6775,11 +7525,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>product_sales</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C41" s="25" t="n">
-        <v>11552.85</v>
+        <v>354.62</v>
       </c>
     </row>
     <row r="42" ht="12" customHeight="1">
@@ -6790,7 +7540,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>shopify_us</t>
+          <t>product_sales</t>
         </is>
       </c>
       <c r="C42" s="25" t="n">
@@ -6800,37 +7550,37 @@
     <row r="43" ht="12" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>202608</t>
+          <t>202607</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>shopify_us</t>
         </is>
       </c>
       <c r="C43" s="25" t="n">
-        <v>0</v>
+        <v>11552.85</v>
       </c>
     </row>
     <row r="44" ht="12" customHeight="1">
       <c r="A44" t="inlineStr">
         <is>
-          <t>202609</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="C44" s="25" t="n">
-        <v>0</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="45" ht="12" customHeight="1">
       <c r="A45" t="inlineStr">
         <is>
-          <t>202610</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -6839,36 +7589,171 @@
         </is>
       </c>
       <c r="C45" s="25" t="n">
-        <v>0</v>
+        <v>215.42</v>
       </c>
     </row>
     <row r="46" ht="12" customHeight="1">
       <c r="A46" t="inlineStr">
         <is>
-          <t>202611</t>
+          <t>202608</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>manufacturing</t>
+          <t>payment_fees</t>
         </is>
       </c>
       <c r="C46" s="25" t="n">
-        <v>0</v>
+        <v>238.45</v>
       </c>
     </row>
     <row r="47" ht="12" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>product_sales</t>
+        </is>
+      </c>
+      <c r="C47" s="25" t="n">
+        <v>8039.34</v>
+      </c>
+    </row>
+    <row r="48" ht="12" customHeight="1">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>202608</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>shopify_us</t>
+        </is>
+      </c>
+      <c r="C48" s="25" t="n">
+        <v>8039.34</v>
+      </c>
+    </row>
+    <row r="49" ht="12" customHeight="1">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+      <c r="C49" s="25" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="50" ht="12" customHeight="1">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C50" s="25" t="n">
+        <v>15.19</v>
+      </c>
+    </row>
+    <row r="51" ht="12" customHeight="1">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>payment_fees</t>
+        </is>
+      </c>
+      <c r="C51" s="25" t="n">
+        <v>37.48</v>
+      </c>
+    </row>
+    <row r="52" ht="12" customHeight="1">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>product_sales</t>
+        </is>
+      </c>
+      <c r="C52" s="25" t="n">
+        <v>1202.61</v>
+      </c>
+    </row>
+    <row r="53" ht="12" customHeight="1">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>202609</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>shopify_us</t>
+        </is>
+      </c>
+      <c r="C53" s="25" t="n">
+        <v>1202.61</v>
+      </c>
+    </row>
+    <row r="54" ht="12" customHeight="1">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C54" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" ht="12" customHeight="1">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>202611</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>manufacturing</t>
+        </is>
+      </c>
+      <c r="C55" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" ht="12" customHeight="1">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>202612</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>manufacturing</t>
         </is>
       </c>
-      <c r="C47" s="25" t="n">
+      <c r="C56" s="25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7100,7 +7985,7 @@
         </is>
       </c>
       <c r="C14" s="26" t="n">
-        <v>0.85715</v>
+        <v>0.85573</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -7115,7 +8000,7 @@
         </is>
       </c>
       <c r="C15" s="26" t="n">
-        <v>1.1476</v>
+        <v>1.1485</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1">
@@ -7130,7 +8015,7 @@
         </is>
       </c>
       <c r="C16" s="26" t="n">
-        <v>0.85715</v>
+        <v>0.85648</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1">
@@ -7145,7 +8030,7 @@
         </is>
       </c>
       <c r="C17" s="26" t="n">
-        <v>1.1476</v>
+        <v>1.1596</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
@@ -7160,7 +8045,7 @@
         </is>
       </c>
       <c r="C18" s="26" t="n">
-        <v>0.85715</v>
+        <v>0.86055</v>
       </c>
     </row>
     <row r="19" ht="12" customHeight="1">
@@ -7175,7 +8060,7 @@
         </is>
       </c>
       <c r="C19" s="26" t="n">
-        <v>1.1476</v>
+        <v>1.1615</v>
       </c>
     </row>
     <row r="20" ht="12" customHeight="1">
@@ -7190,7 +8075,7 @@
         </is>
       </c>
       <c r="C20" s="26" t="n">
-        <v>0.85715</v>
+        <v>0.86055</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
@@ -7205,7 +8090,7 @@
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>1.1476</v>
+        <v>1.1615</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1">
@@ -7220,7 +8105,7 @@
         </is>
       </c>
       <c r="C22" s="26" t="n">
-        <v>0.85715</v>
+        <v>0.86055</v>
       </c>
     </row>
     <row r="23" ht="12" customHeight="1">
@@ -7235,7 +8120,7 @@
         </is>
       </c>
       <c r="C23" s="26" t="n">
-        <v>1.1476</v>
+        <v>1.1615</v>
       </c>
     </row>
     <row r="24" ht="12" customHeight="1">
@@ -7250,7 +8135,7 @@
         </is>
       </c>
       <c r="C24" s="26" t="n">
-        <v>0.85715</v>
+        <v>0.86055</v>
       </c>
     </row>
     <row r="25" ht="12" customHeight="1">
@@ -7265,7 +8150,7 @@
         </is>
       </c>
       <c r="C25" s="26" t="n">
-        <v>1.1476</v>
+        <v>1.1615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>